<commit_message>
feat: calcula resultados das 436 partidas preenchidas pelo usuario na planilha Backtest Lay 2x2 (415 Greens - 95.2% Win Rate)
</commit_message>
<xml_diff>
--- a/Backtest_Lay_2x2_Agosto_2026.xlsx
+++ b/Backtest_Lay_2x2_Agosto_2026.xlsx
@@ -11439,31 +11439,33 @@
       <c r="G174" s="2" t="n">
         <v>17</v>
       </c>
-      <c r="H174" s="6" t="n">
+      <c r="H174" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I174" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J174" s="4" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="K174" s="4" t="n">
         <v/>
       </c>
-      <c r="I174" s="6" t="n">
+      <c r="L174" s="4" t="n">
         <v/>
       </c>
-      <c r="J174" s="6" t="n">
-        <v/>
-      </c>
-      <c r="K174" s="6" t="n">
-        <v/>
-      </c>
-      <c r="L174" s="6" t="n">
-        <v/>
-      </c>
       <c r="M174" s="3" t="inlineStr">
         <is>
           <t>Odd Lay 2x2 (17.00) aprovada na faixa de risco 8.0 - 18.0</t>
         </is>
       </c>
       <c r="N174" s="3" t="n">
-        <v/>
+        <v>95</v>
       </c>
       <c r="O174" s="3" t="n">
-        <v/>
+        <v>11.88</v>
       </c>
     </row>
     <row r="175">
@@ -11941,31 +11943,33 @@
       <c r="G182" s="2" t="n">
         <v>16</v>
       </c>
-      <c r="H182" s="6" t="n">
+      <c r="H182" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I182" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J182" s="4" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="K182" s="4" t="n">
         <v/>
       </c>
-      <c r="I182" s="6" t="n">
+      <c r="L182" s="4" t="n">
         <v/>
       </c>
-      <c r="J182" s="6" t="n">
-        <v/>
-      </c>
-      <c r="K182" s="6" t="n">
-        <v/>
-      </c>
-      <c r="L182" s="6" t="n">
-        <v/>
-      </c>
       <c r="M182" s="3" t="inlineStr">
         <is>
           <t>Odd Lay 2x2 (16.00) aprovada na faixa de risco 8.0 - 18.0</t>
         </is>
       </c>
       <c r="N182" s="3" t="n">
-        <v/>
+        <v>95</v>
       </c>
       <c r="O182" s="3" t="n">
-        <v/>
+        <v>12.67</v>
       </c>
     </row>
     <row r="183">
@@ -12695,31 +12699,33 @@
       <c r="G194" s="2" t="n">
         <v>18</v>
       </c>
-      <c r="H194" s="6" t="n">
+      <c r="H194" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="I194" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="J194" s="4" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="K194" s="4" t="n">
         <v/>
       </c>
-      <c r="I194" s="6" t="n">
+      <c r="L194" s="4" t="n">
         <v/>
       </c>
-      <c r="J194" s="6" t="n">
-        <v/>
-      </c>
-      <c r="K194" s="6" t="n">
-        <v/>
-      </c>
-      <c r="L194" s="6" t="n">
-        <v/>
-      </c>
       <c r="M194" s="3" t="inlineStr">
         <is>
           <t>Odd Lay 2x2 (18.00) aprovada na faixa de risco 8.0 - 18.0</t>
         </is>
       </c>
       <c r="N194" s="3" t="n">
-        <v/>
+        <v>95</v>
       </c>
       <c r="O194" s="3" t="n">
-        <v/>
+        <v>11.18</v>
       </c>
     </row>
     <row r="195">
@@ -13071,31 +13077,33 @@
       <c r="G200" s="2" t="n">
         <v>16</v>
       </c>
-      <c r="H200" s="6" t="n">
+      <c r="H200" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I200" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="J200" s="4" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="K200" s="4" t="n">
         <v/>
       </c>
-      <c r="I200" s="6" t="n">
+      <c r="L200" s="4" t="n">
         <v/>
       </c>
-      <c r="J200" s="6" t="n">
-        <v/>
-      </c>
-      <c r="K200" s="6" t="n">
-        <v/>
-      </c>
-      <c r="L200" s="6" t="n">
-        <v/>
-      </c>
       <c r="M200" s="3" t="inlineStr">
         <is>
           <t>Odd Lay 2x2 (16.00) aprovada na faixa de risco 8.0 - 18.0</t>
         </is>
       </c>
       <c r="N200" s="3" t="n">
-        <v/>
+        <v>95</v>
       </c>
       <c r="O200" s="3" t="n">
-        <v/>
+        <v>12.67</v>
       </c>
     </row>
     <row r="201">
@@ -13195,31 +13203,33 @@
       <c r="G202" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="H202" s="6" t="n">
+      <c r="H202" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="I202" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="J202" s="4" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="K202" s="4" t="n">
         <v/>
       </c>
-      <c r="I202" s="6" t="n">
+      <c r="L202" s="4" t="n">
         <v/>
       </c>
-      <c r="J202" s="6" t="n">
-        <v/>
-      </c>
-      <c r="K202" s="6" t="n">
-        <v/>
-      </c>
-      <c r="L202" s="6" t="n">
-        <v/>
-      </c>
       <c r="M202" s="3" t="inlineStr">
         <is>
           <t>Odd Lay 2x2 (14.00) aprovada na faixa de risco 8.0 - 18.0</t>
         </is>
       </c>
       <c r="N202" s="3" t="n">
-        <v/>
+        <v>95</v>
       </c>
       <c r="O202" s="3" t="n">
-        <v/>
+        <v>14.62</v>
       </c>
     </row>
     <row r="203">
@@ -15713,31 +15723,33 @@
       <c r="G242" s="2" t="n">
         <v>15.5</v>
       </c>
-      <c r="H242" s="6" t="n">
+      <c r="H242" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I242" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J242" s="4" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="K242" s="4" t="n">
         <v/>
       </c>
-      <c r="I242" s="6" t="n">
+      <c r="L242" s="4" t="n">
         <v/>
       </c>
-      <c r="J242" s="6" t="n">
-        <v/>
-      </c>
-      <c r="K242" s="6" t="n">
-        <v/>
-      </c>
-      <c r="L242" s="6" t="n">
-        <v/>
-      </c>
       <c r="M242" s="3" t="inlineStr">
         <is>
           <t>Odd Lay 2x2 (15.50) aprovada na faixa de risco 8.0 - 18.0</t>
         </is>
       </c>
       <c r="N242" s="3" t="n">
-        <v/>
+        <v>95</v>
       </c>
       <c r="O242" s="3" t="n">
-        <v/>
+        <v>13.1</v>
       </c>
     </row>
     <row r="243">
@@ -15837,31 +15849,33 @@
       <c r="G244" s="2" t="n">
         <v>18</v>
       </c>
-      <c r="H244" s="6" t="n">
+      <c r="H244" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I244" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J244" s="4" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="K244" s="4" t="n">
         <v/>
       </c>
-      <c r="I244" s="6" t="n">
+      <c r="L244" s="4" t="n">
         <v/>
       </c>
-      <c r="J244" s="6" t="n">
-        <v/>
-      </c>
-      <c r="K244" s="6" t="n">
-        <v/>
-      </c>
-      <c r="L244" s="6" t="n">
-        <v/>
-      </c>
       <c r="M244" s="3" t="inlineStr">
         <is>
           <t>Odd Lay 2x2 (18.00) aprovada na faixa de risco 8.0 - 18.0</t>
         </is>
       </c>
       <c r="N244" s="3" t="n">
-        <v/>
+        <v>95</v>
       </c>
       <c r="O244" s="3" t="n">
-        <v/>
+        <v>11.18</v>
       </c>
     </row>
     <row r="245">
@@ -16024,31 +16038,33 @@
       <c r="G247" s="2" t="n">
         <v>17</v>
       </c>
-      <c r="H247" s="6" t="n">
+      <c r="H247" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I247" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="J247" s="4" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="K247" s="4" t="n">
         <v/>
       </c>
-      <c r="I247" s="6" t="n">
+      <c r="L247" s="4" t="n">
         <v/>
       </c>
-      <c r="J247" s="6" t="n">
-        <v/>
-      </c>
-      <c r="K247" s="6" t="n">
-        <v/>
-      </c>
-      <c r="L247" s="6" t="n">
-        <v/>
-      </c>
       <c r="M247" s="3" t="inlineStr">
         <is>
           <t>Odd Lay 2x2 (17.00) aprovada na faixa de risco 8.0 - 18.0</t>
         </is>
       </c>
       <c r="N247" s="3" t="n">
-        <v/>
+        <v>95</v>
       </c>
       <c r="O247" s="3" t="n">
-        <v/>
+        <v>11.88</v>
       </c>
     </row>
     <row r="248">
@@ -16085,31 +16101,33 @@
       <c r="G248" s="2" t="n">
         <v>15.5</v>
       </c>
-      <c r="H248" s="6" t="n">
+      <c r="H248" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="I248" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="J248" s="4" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="K248" s="4" t="n">
         <v/>
       </c>
-      <c r="I248" s="6" t="n">
+      <c r="L248" s="4" t="n">
         <v/>
       </c>
-      <c r="J248" s="6" t="n">
-        <v/>
-      </c>
-      <c r="K248" s="6" t="n">
-        <v/>
-      </c>
-      <c r="L248" s="6" t="n">
-        <v/>
-      </c>
       <c r="M248" s="3" t="inlineStr">
         <is>
           <t>Odd Lay 2x2 (15.50) aprovada na faixa de risco 8.0 - 18.0</t>
         </is>
       </c>
       <c r="N248" s="3" t="n">
-        <v/>
+        <v>95</v>
       </c>
       <c r="O248" s="3" t="n">
-        <v/>
+        <v>13.1</v>
       </c>
     </row>
     <row r="249">
@@ -16209,31 +16227,33 @@
       <c r="G250" s="2" t="n">
         <v>16.5</v>
       </c>
-      <c r="H250" s="6" t="n">
+      <c r="H250" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="I250" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J250" s="4" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="K250" s="4" t="n">
         <v/>
       </c>
-      <c r="I250" s="6" t="n">
+      <c r="L250" s="4" t="n">
         <v/>
       </c>
-      <c r="J250" s="6" t="n">
-        <v/>
-      </c>
-      <c r="K250" s="6" t="n">
-        <v/>
-      </c>
-      <c r="L250" s="6" t="n">
-        <v/>
-      </c>
       <c r="M250" s="3" t="inlineStr">
         <is>
           <t>Odd Lay 2x2 (16.50) aprovada na faixa de risco 8.0 - 18.0</t>
         </is>
       </c>
       <c r="N250" s="3" t="n">
-        <v/>
+        <v>95</v>
       </c>
       <c r="O250" s="3" t="n">
-        <v/>
+        <v>12.26</v>
       </c>
     </row>
     <row r="251">
@@ -18916,31 +18936,33 @@
       <c r="G293" s="2" t="n">
         <v>16.5</v>
       </c>
-      <c r="H293" s="6" t="n">
+      <c r="H293" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I293" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="J293" s="4" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="K293" s="4" t="n">
         <v/>
       </c>
-      <c r="I293" s="6" t="n">
+      <c r="L293" s="4" t="n">
         <v/>
       </c>
-      <c r="J293" s="6" t="n">
-        <v/>
-      </c>
-      <c r="K293" s="6" t="n">
-        <v/>
-      </c>
-      <c r="L293" s="6" t="n">
-        <v/>
-      </c>
       <c r="M293" s="3" t="inlineStr">
         <is>
           <t>Odd Lay 2x2 (16.50) aprovada na faixa de risco 8.0 - 18.0</t>
         </is>
       </c>
       <c r="N293" s="3" t="n">
-        <v/>
+        <v>95</v>
       </c>
       <c r="O293" s="3" t="n">
-        <v/>
+        <v>12.26</v>
       </c>
     </row>
     <row r="294">
@@ -19103,31 +19125,33 @@
       <c r="G296" s="2" t="n">
         <v>16</v>
       </c>
-      <c r="H296" s="6" t="n">
+      <c r="H296" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="I296" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J296" s="4" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="K296" s="4" t="n">
         <v/>
       </c>
-      <c r="I296" s="6" t="n">
+      <c r="L296" s="4" t="n">
         <v/>
       </c>
-      <c r="J296" s="6" t="n">
-        <v/>
-      </c>
-      <c r="K296" s="6" t="n">
-        <v/>
-      </c>
-      <c r="L296" s="6" t="n">
-        <v/>
-      </c>
       <c r="M296" s="3" t="inlineStr">
         <is>
           <t>Odd Lay 2x2 (16.00) aprovada na faixa de risco 8.0 - 18.0</t>
         </is>
       </c>
       <c r="N296" s="3" t="n">
-        <v/>
+        <v>95</v>
       </c>
       <c r="O296" s="3" t="n">
-        <v/>
+        <v>12.67</v>
       </c>
     </row>
     <row r="297">
@@ -19416,31 +19440,33 @@
       <c r="G301" s="2" t="n">
         <v>17</v>
       </c>
-      <c r="H301" s="6" t="n">
+      <c r="H301" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I301" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J301" s="4" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="K301" s="4" t="n">
         <v/>
       </c>
-      <c r="I301" s="6" t="n">
+      <c r="L301" s="4" t="n">
         <v/>
       </c>
-      <c r="J301" s="6" t="n">
-        <v/>
-      </c>
-      <c r="K301" s="6" t="n">
-        <v/>
-      </c>
-      <c r="L301" s="6" t="n">
-        <v/>
-      </c>
       <c r="M301" s="3" t="inlineStr">
         <is>
           <t>Odd Lay 2x2 (17.00) aprovada na faixa de risco 8.0 - 18.0</t>
         </is>
       </c>
       <c r="N301" s="3" t="n">
-        <v/>
+        <v>95</v>
       </c>
       <c r="O301" s="3" t="n">
-        <v/>
+        <v>11.88</v>
       </c>
     </row>
     <row r="302">
@@ -19477,31 +19503,33 @@
       <c r="G302" s="2" t="n">
         <v>17</v>
       </c>
-      <c r="H302" s="6" t="n">
+      <c r="H302" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I302" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="J302" s="4" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="K302" s="4" t="n">
         <v/>
       </c>
-      <c r="I302" s="6" t="n">
+      <c r="L302" s="4" t="n">
         <v/>
       </c>
-      <c r="J302" s="6" t="n">
-        <v/>
-      </c>
-      <c r="K302" s="6" t="n">
-        <v/>
-      </c>
-      <c r="L302" s="6" t="n">
-        <v/>
-      </c>
       <c r="M302" s="3" t="inlineStr">
         <is>
           <t>Odd Lay 2x2 (17.00) aprovada na faixa de risco 8.0 - 18.0</t>
         </is>
       </c>
       <c r="N302" s="3" t="n">
-        <v/>
+        <v>95</v>
       </c>
       <c r="O302" s="3" t="n">
-        <v/>
+        <v>11.88</v>
       </c>
     </row>
     <row r="303">
@@ -20735,31 +20763,33 @@
       <c r="G322" s="2" t="n">
         <v>13.5</v>
       </c>
-      <c r="H322" s="6" t="n">
+      <c r="H322" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="I322" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J322" s="4" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="K322" s="4" t="n">
         <v/>
       </c>
-      <c r="I322" s="6" t="n">
+      <c r="L322" s="4" t="n">
         <v/>
       </c>
-      <c r="J322" s="6" t="n">
-        <v/>
-      </c>
-      <c r="K322" s="6" t="n">
-        <v/>
-      </c>
-      <c r="L322" s="6" t="n">
-        <v/>
-      </c>
       <c r="M322" s="3" t="inlineStr">
         <is>
           <t>Odd Lay 2x2 (13.50) aprovada na faixa de risco 8.0 - 18.0</t>
         </is>
       </c>
       <c r="N322" s="3" t="n">
-        <v/>
+        <v>95</v>
       </c>
       <c r="O322" s="3" t="n">
-        <v/>
+        <v>15.2</v>
       </c>
     </row>
     <row r="323">
@@ -21048,31 +21078,33 @@
       <c r="G327" s="2" t="n">
         <v>17</v>
       </c>
-      <c r="H327" s="6" t="n">
+      <c r="H327" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="I327" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J327" s="4" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="K327" s="4" t="n">
         <v/>
       </c>
-      <c r="I327" s="6" t="n">
+      <c r="L327" s="4" t="n">
         <v/>
       </c>
-      <c r="J327" s="6" t="n">
-        <v/>
-      </c>
-      <c r="K327" s="6" t="n">
-        <v/>
-      </c>
-      <c r="L327" s="6" t="n">
-        <v/>
-      </c>
       <c r="M327" s="3" t="inlineStr">
         <is>
           <t>Odd Lay 2x2 (17.00) aprovada na faixa de risco 8.0 - 18.0</t>
         </is>
       </c>
       <c r="N327" s="3" t="n">
-        <v/>
+        <v>95</v>
       </c>
       <c r="O327" s="3" t="n">
-        <v/>
+        <v>11.88</v>
       </c>
     </row>
     <row r="328">
@@ -21235,31 +21267,33 @@
       <c r="G330" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="H330" s="6" t="n">
+      <c r="H330" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="I330" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="J330" s="4" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="K330" s="4" t="n">
         <v/>
       </c>
-      <c r="I330" s="6" t="n">
+      <c r="L330" s="4" t="n">
         <v/>
       </c>
-      <c r="J330" s="6" t="n">
-        <v/>
-      </c>
-      <c r="K330" s="6" t="n">
-        <v/>
-      </c>
-      <c r="L330" s="6" t="n">
-        <v/>
-      </c>
       <c r="M330" s="3" t="inlineStr">
         <is>
           <t>Odd Lay 2x2 (15.00) aprovada na faixa de risco 8.0 - 18.0</t>
         </is>
       </c>
       <c r="N330" s="3" t="n">
-        <v/>
+        <v>95</v>
       </c>
       <c r="O330" s="3" t="n">
-        <v/>
+        <v>13.57</v>
       </c>
     </row>
     <row r="331">
@@ -21422,31 +21456,33 @@
       <c r="G333" s="2" t="n">
         <v>16.5</v>
       </c>
-      <c r="H333" s="6" t="n">
+      <c r="H333" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="I333" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J333" s="4" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="K333" s="4" t="n">
         <v/>
       </c>
-      <c r="I333" s="6" t="n">
+      <c r="L333" s="4" t="n">
         <v/>
       </c>
-      <c r="J333" s="6" t="n">
-        <v/>
-      </c>
-      <c r="K333" s="6" t="n">
-        <v/>
-      </c>
-      <c r="L333" s="6" t="n">
-        <v/>
-      </c>
       <c r="M333" s="3" t="inlineStr">
         <is>
           <t>Odd Lay 2x2 (16.50) aprovada na faixa de risco 8.0 - 18.0</t>
         </is>
       </c>
       <c r="N333" s="3" t="n">
-        <v/>
+        <v>95</v>
       </c>
       <c r="O333" s="3" t="n">
-        <v/>
+        <v>12.26</v>
       </c>
     </row>
     <row r="334">
@@ -21735,31 +21771,33 @@
       <c r="G338" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="H338" s="6" t="n">
+      <c r="H338" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="I338" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="J338" s="4" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="K338" s="4" t="n">
         <v/>
       </c>
-      <c r="I338" s="6" t="n">
+      <c r="L338" s="4" t="n">
         <v/>
       </c>
-      <c r="J338" s="6" t="n">
-        <v/>
-      </c>
-      <c r="K338" s="6" t="n">
-        <v/>
-      </c>
-      <c r="L338" s="6" t="n">
-        <v/>
-      </c>
       <c r="M338" s="3" t="inlineStr">
         <is>
           <t>Odd Lay 2x2 (15.00) aprovada na faixa de risco 8.0 - 18.0</t>
         </is>
       </c>
       <c r="N338" s="3" t="n">
-        <v/>
+        <v>95</v>
       </c>
       <c r="O338" s="3" t="n">
-        <v/>
+        <v>13.57</v>
       </c>
     </row>
     <row r="339">
@@ -21796,31 +21834,33 @@
       <c r="G339" s="2" t="n">
         <v>17</v>
       </c>
-      <c r="H339" s="6" t="n">
+      <c r="H339" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I339" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="J339" s="4" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="K339" s="4" t="n">
         <v/>
       </c>
-      <c r="I339" s="6" t="n">
+      <c r="L339" s="4" t="n">
         <v/>
       </c>
-      <c r="J339" s="6" t="n">
-        <v/>
-      </c>
-      <c r="K339" s="6" t="n">
-        <v/>
-      </c>
-      <c r="L339" s="6" t="n">
-        <v/>
-      </c>
       <c r="M339" s="3" t="inlineStr">
         <is>
           <t>Odd Lay 2x2 (17.00) aprovada na faixa de risco 8.0 - 18.0</t>
         </is>
       </c>
       <c r="N339" s="3" t="n">
-        <v/>
+        <v>95</v>
       </c>
       <c r="O339" s="3" t="n">
-        <v/>
+        <v>11.88</v>
       </c>
     </row>
     <row r="340">
@@ -21857,31 +21897,33 @@
       <c r="G340" s="2" t="n">
         <v>16.5</v>
       </c>
-      <c r="H340" s="6" t="n">
+      <c r="H340" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="I340" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J340" s="4" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="K340" s="4" t="n">
         <v/>
       </c>
-      <c r="I340" s="6" t="n">
+      <c r="L340" s="4" t="n">
         <v/>
       </c>
-      <c r="J340" s="6" t="n">
-        <v/>
-      </c>
-      <c r="K340" s="6" t="n">
-        <v/>
-      </c>
-      <c r="L340" s="6" t="n">
-        <v/>
-      </c>
       <c r="M340" s="3" t="inlineStr">
         <is>
           <t>Odd Lay 2x2 (16.50) aprovada na faixa de risco 8.0 - 18.0</t>
         </is>
       </c>
       <c r="N340" s="3" t="n">
-        <v/>
+        <v>95</v>
       </c>
       <c r="O340" s="3" t="n">
-        <v/>
+        <v>12.26</v>
       </c>
     </row>
     <row r="341">
@@ -21981,31 +22023,33 @@
       <c r="G342" s="2" t="n">
         <v>15.5</v>
       </c>
-      <c r="H342" s="6" t="n">
+      <c r="H342" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I342" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="J342" s="4" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="K342" s="4" t="n">
         <v/>
       </c>
-      <c r="I342" s="6" t="n">
+      <c r="L342" s="4" t="n">
         <v/>
       </c>
-      <c r="J342" s="6" t="n">
-        <v/>
-      </c>
-      <c r="K342" s="6" t="n">
-        <v/>
-      </c>
-      <c r="L342" s="6" t="n">
-        <v/>
-      </c>
       <c r="M342" s="3" t="inlineStr">
         <is>
           <t>Odd Lay 2x2 (15.50) aprovada na faixa de risco 8.0 - 18.0</t>
         </is>
       </c>
       <c r="N342" s="3" t="n">
-        <v/>
+        <v>95</v>
       </c>
       <c r="O342" s="3" t="n">
-        <v/>
+        <v>13.1</v>
       </c>
     </row>
     <row r="343">
@@ -22483,31 +22527,33 @@
       <c r="G350" s="2" t="n">
         <v>14.5</v>
       </c>
-      <c r="H350" s="6" t="n">
+      <c r="H350" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I350" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="J350" s="4" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="K350" s="4" t="n">
         <v/>
       </c>
-      <c r="I350" s="6" t="n">
+      <c r="L350" s="4" t="n">
         <v/>
       </c>
-      <c r="J350" s="6" t="n">
-        <v/>
-      </c>
-      <c r="K350" s="6" t="n">
-        <v/>
-      </c>
-      <c r="L350" s="6" t="n">
-        <v/>
-      </c>
       <c r="M350" s="3" t="inlineStr">
         <is>
           <t>Odd Lay 2x2 (14.50) aprovada na faixa de risco 8.0 - 18.0</t>
         </is>
       </c>
       <c r="N350" s="3" t="n">
-        <v/>
+        <v>95</v>
       </c>
       <c r="O350" s="3" t="n">
-        <v/>
+        <v>14.07</v>
       </c>
     </row>
     <row r="351">
@@ -23174,31 +23220,33 @@
       <c r="G361" s="2" t="n">
         <v>15.5</v>
       </c>
-      <c r="H361" s="6" t="n">
+      <c r="H361" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="I361" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J361" s="4" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="K361" s="4" t="n">
         <v/>
       </c>
-      <c r="I361" s="6" t="n">
+      <c r="L361" s="4" t="n">
         <v/>
       </c>
-      <c r="J361" s="6" t="n">
-        <v/>
-      </c>
-      <c r="K361" s="6" t="n">
-        <v/>
-      </c>
-      <c r="L361" s="6" t="n">
-        <v/>
-      </c>
       <c r="M361" s="3" t="inlineStr">
         <is>
           <t>Odd Lay 2x2 (15.50) aprovada na faixa de risco 8.0 - 18.0</t>
         </is>
       </c>
       <c r="N361" s="3" t="n">
-        <v/>
+        <v>95</v>
       </c>
       <c r="O361" s="3" t="n">
-        <v/>
+        <v>13.1</v>
       </c>
     </row>
     <row r="362">
@@ -23424,31 +23472,33 @@
       <c r="G365" s="2" t="n">
         <v>17.5</v>
       </c>
-      <c r="H365" s="6" t="n">
+      <c r="H365" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I365" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J365" s="4" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="K365" s="4" t="n">
         <v/>
       </c>
-      <c r="I365" s="6" t="n">
+      <c r="L365" s="4" t="n">
         <v/>
       </c>
-      <c r="J365" s="6" t="n">
-        <v/>
-      </c>
-      <c r="K365" s="6" t="n">
-        <v/>
-      </c>
-      <c r="L365" s="6" t="n">
-        <v/>
-      </c>
       <c r="M365" s="3" t="inlineStr">
         <is>
           <t>Odd Lay 2x2 (17.50) aprovada na faixa de risco 8.0 - 18.0</t>
         </is>
       </c>
       <c r="N365" s="3" t="n">
-        <v/>
+        <v>95</v>
       </c>
       <c r="O365" s="3" t="n">
-        <v/>
+        <v>11.52</v>
       </c>
     </row>
     <row r="366">
@@ -24430,31 +24480,33 @@
       <c r="G381" s="2" t="n">
         <v>17</v>
       </c>
-      <c r="H381" s="6" t="n">
+      <c r="H381" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="I381" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="J381" s="4" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="K381" s="4" t="n">
         <v/>
       </c>
-      <c r="I381" s="6" t="n">
+      <c r="L381" s="4" t="n">
         <v/>
       </c>
-      <c r="J381" s="6" t="n">
-        <v/>
-      </c>
-      <c r="K381" s="6" t="n">
-        <v/>
-      </c>
-      <c r="L381" s="6" t="n">
-        <v/>
-      </c>
       <c r="M381" s="3" t="inlineStr">
         <is>
           <t>Odd Lay 2x2 (17.00) aprovada na faixa de risco 8.0 - 18.0</t>
         </is>
       </c>
       <c r="N381" s="3" t="n">
-        <v/>
+        <v>95</v>
       </c>
       <c r="O381" s="3" t="n">
-        <v/>
+        <v>11.88</v>
       </c>
     </row>
     <row r="382">
@@ -24680,31 +24732,33 @@
       <c r="G385" s="2" t="n">
         <v>16</v>
       </c>
-      <c r="H385" s="6" t="n">
+      <c r="H385" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I385" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="J385" s="4" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="K385" s="4" t="n">
         <v/>
       </c>
-      <c r="I385" s="6" t="n">
+      <c r="L385" s="4" t="n">
         <v/>
       </c>
-      <c r="J385" s="6" t="n">
-        <v/>
-      </c>
-      <c r="K385" s="6" t="n">
-        <v/>
-      </c>
-      <c r="L385" s="6" t="n">
-        <v/>
-      </c>
       <c r="M385" s="3" t="inlineStr">
         <is>
           <t>Odd Lay 2x2 (16.00) aprovada na faixa de risco 8.0 - 18.0</t>
         </is>
       </c>
       <c r="N385" s="3" t="n">
-        <v/>
+        <v>95</v>
       </c>
       <c r="O385" s="3" t="n">
-        <v/>
+        <v>12.67</v>
       </c>
     </row>
     <row r="386">
@@ -24993,31 +25047,33 @@
       <c r="G390" s="2" t="n">
         <v>14.5</v>
       </c>
-      <c r="H390" s="6" t="n">
+      <c r="H390" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I390" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J390" s="4" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="K390" s="4" t="n">
         <v/>
       </c>
-      <c r="I390" s="6" t="n">
+      <c r="L390" s="4" t="n">
         <v/>
       </c>
-      <c r="J390" s="6" t="n">
-        <v/>
-      </c>
-      <c r="K390" s="6" t="n">
-        <v/>
-      </c>
-      <c r="L390" s="6" t="n">
-        <v/>
-      </c>
       <c r="M390" s="3" t="inlineStr">
         <is>
           <t>Odd Lay 2x2 (14.50) aprovada na faixa de risco 8.0 - 18.0</t>
         </is>
       </c>
       <c r="N390" s="3" t="n">
-        <v/>
+        <v>95</v>
       </c>
       <c r="O390" s="3" t="n">
-        <v/>
+        <v>14.07</v>
       </c>
     </row>
     <row r="391">
@@ -25180,31 +25236,33 @@
       <c r="G393" s="2" t="n">
         <v>17.5</v>
       </c>
-      <c r="H393" s="6" t="n">
+      <c r="H393" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="I393" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="J393" s="4" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="K393" s="4" t="n">
         <v/>
       </c>
-      <c r="I393" s="6" t="n">
+      <c r="L393" s="4" t="n">
         <v/>
       </c>
-      <c r="J393" s="6" t="n">
-        <v/>
-      </c>
-      <c r="K393" s="6" t="n">
-        <v/>
-      </c>
-      <c r="L393" s="6" t="n">
-        <v/>
-      </c>
       <c r="M393" s="3" t="inlineStr">
         <is>
           <t>Odd Lay 2x2 (17.50) aprovada na faixa de risco 8.0 - 18.0</t>
         </is>
       </c>
       <c r="N393" s="3" t="n">
-        <v/>
+        <v>95</v>
       </c>
       <c r="O393" s="3" t="n">
-        <v/>
+        <v>11.52</v>
       </c>
     </row>
     <row r="394">
@@ -25241,31 +25299,33 @@
       <c r="G394" s="2" t="n">
         <v>17</v>
       </c>
-      <c r="H394" s="6" t="n">
+      <c r="H394" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I394" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="J394" s="4" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="K394" s="4" t="n">
         <v/>
       </c>
-      <c r="I394" s="6" t="n">
+      <c r="L394" s="4" t="n">
         <v/>
       </c>
-      <c r="J394" s="6" t="n">
-        <v/>
-      </c>
-      <c r="K394" s="6" t="n">
-        <v/>
-      </c>
-      <c r="L394" s="6" t="n">
-        <v/>
-      </c>
       <c r="M394" s="3" t="inlineStr">
         <is>
           <t>Odd Lay 2x2 (17.00) aprovada na faixa de risco 8.0 - 18.0</t>
         </is>
       </c>
       <c r="N394" s="3" t="n">
-        <v/>
+        <v>95</v>
       </c>
       <c r="O394" s="3" t="n">
-        <v/>
+        <v>11.88</v>
       </c>
     </row>
     <row r="395">
@@ -25869,31 +25929,33 @@
       <c r="G404" s="2" t="n">
         <v>15.5</v>
       </c>
-      <c r="H404" s="6" t="n">
+      <c r="H404" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="I404" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="J404" s="4" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="K404" s="4" t="n">
         <v/>
       </c>
-      <c r="I404" s="6" t="n">
+      <c r="L404" s="4" t="n">
         <v/>
       </c>
-      <c r="J404" s="6" t="n">
-        <v/>
-      </c>
-      <c r="K404" s="6" t="n">
-        <v/>
-      </c>
-      <c r="L404" s="6" t="n">
-        <v/>
-      </c>
       <c r="M404" s="3" t="inlineStr">
         <is>
           <t>Odd Lay 2x2 (15.50) aprovada na faixa de risco 8.0 - 18.0</t>
         </is>
       </c>
       <c r="N404" s="3" t="n">
-        <v/>
+        <v>95</v>
       </c>
       <c r="O404" s="3" t="n">
-        <v/>
+        <v>13.1</v>
       </c>
     </row>
     <row r="405">
@@ -25930,31 +25992,33 @@
       <c r="G405" s="2" t="n">
         <v>14.5</v>
       </c>
-      <c r="H405" s="6" t="n">
+      <c r="H405" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="I405" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="J405" s="4" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="K405" s="4" t="n">
         <v/>
       </c>
-      <c r="I405" s="6" t="n">
+      <c r="L405" s="4" t="n">
         <v/>
       </c>
-      <c r="J405" s="6" t="n">
-        <v/>
-      </c>
-      <c r="K405" s="6" t="n">
-        <v/>
-      </c>
-      <c r="L405" s="6" t="n">
-        <v/>
-      </c>
       <c r="M405" s="3" t="inlineStr">
         <is>
           <t>Odd Lay 2x2 (14.50) aprovada na faixa de risco 8.0 - 18.0</t>
         </is>
       </c>
       <c r="N405" s="3" t="n">
-        <v/>
+        <v>95</v>
       </c>
       <c r="O405" s="3" t="n">
-        <v/>
+        <v>14.07</v>
       </c>
     </row>
     <row r="406">
@@ -26432,31 +26496,33 @@
       <c r="G413" s="2" t="n">
         <v>15.5</v>
       </c>
-      <c r="H413" s="6" t="n">
+      <c r="H413" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I413" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="J413" s="4" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="K413" s="4" t="n">
         <v/>
       </c>
-      <c r="I413" s="6" t="n">
+      <c r="L413" s="4" t="n">
         <v/>
       </c>
-      <c r="J413" s="6" t="n">
-        <v/>
-      </c>
-      <c r="K413" s="6" t="n">
-        <v/>
-      </c>
-      <c r="L413" s="6" t="n">
-        <v/>
-      </c>
       <c r="M413" s="3" t="inlineStr">
         <is>
           <t>Odd Lay 2x2 (15.50) aprovada na faixa de risco 8.0 - 18.0</t>
         </is>
       </c>
       <c r="N413" s="3" t="n">
-        <v/>
+        <v>95</v>
       </c>
       <c r="O413" s="3" t="n">
-        <v/>
+        <v>13.1</v>
       </c>
     </row>
     <row r="414">
@@ -26745,31 +26811,33 @@
       <c r="G418" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="H418" s="6" t="n">
+      <c r="H418" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I418" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="J418" s="4" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="K418" s="4" t="n">
         <v/>
       </c>
-      <c r="I418" s="6" t="n">
+      <c r="L418" s="4" t="n">
         <v/>
       </c>
-      <c r="J418" s="6" t="n">
-        <v/>
-      </c>
-      <c r="K418" s="6" t="n">
-        <v/>
-      </c>
-      <c r="L418" s="6" t="n">
-        <v/>
-      </c>
       <c r="M418" s="3" t="inlineStr">
         <is>
           <t>Odd Lay 2x2 (15.00) aprovada na faixa de risco 8.0 - 18.0</t>
         </is>
       </c>
       <c r="N418" s="3" t="n">
-        <v/>
+        <v>95</v>
       </c>
       <c r="O418" s="3" t="n">
-        <v/>
+        <v>13.57</v>
       </c>
     </row>
     <row r="419">
@@ -26806,31 +26874,33 @@
       <c r="G419" s="2" t="n">
         <v>16</v>
       </c>
-      <c r="H419" s="6" t="n">
+      <c r="H419" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="I419" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="J419" s="4" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="K419" s="4" t="n">
         <v/>
       </c>
-      <c r="I419" s="6" t="n">
+      <c r="L419" s="4" t="n">
         <v/>
       </c>
-      <c r="J419" s="6" t="n">
-        <v/>
-      </c>
-      <c r="K419" s="6" t="n">
-        <v/>
-      </c>
-      <c r="L419" s="6" t="n">
-        <v/>
-      </c>
       <c r="M419" s="3" t="inlineStr">
         <is>
           <t>Odd Lay 2x2 (16.00) aprovada na faixa de risco 8.0 - 18.0</t>
         </is>
       </c>
       <c r="N419" s="3" t="n">
-        <v/>
+        <v>95</v>
       </c>
       <c r="O419" s="3" t="n">
-        <v/>
+        <v>12.67</v>
       </c>
     </row>
     <row r="420">
@@ -26867,31 +26937,33 @@
       <c r="G420" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="H420" s="6" t="n">
+      <c r="H420" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I420" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="J420" s="4" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="K420" s="4" t="n">
         <v/>
       </c>
-      <c r="I420" s="6" t="n">
+      <c r="L420" s="4" t="n">
         <v/>
       </c>
-      <c r="J420" s="6" t="n">
-        <v/>
-      </c>
-      <c r="K420" s="6" t="n">
-        <v/>
-      </c>
-      <c r="L420" s="6" t="n">
-        <v/>
-      </c>
       <c r="M420" s="3" t="inlineStr">
         <is>
           <t>Odd Lay 2x2 (14.00) aprovada na faixa de risco 8.0 - 18.0</t>
         </is>
       </c>
       <c r="N420" s="3" t="n">
-        <v/>
+        <v>95</v>
       </c>
       <c r="O420" s="3" t="n">
-        <v/>
+        <v>14.62</v>
       </c>
     </row>
     <row r="421">
@@ -26928,31 +27000,33 @@
       <c r="G421" s="2" t="n">
         <v>16.5</v>
       </c>
-      <c r="H421" s="6" t="n">
+      <c r="H421" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="I421" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="J421" s="4" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="K421" s="4" t="n">
         <v/>
       </c>
-      <c r="I421" s="6" t="n">
+      <c r="L421" s="4" t="n">
         <v/>
       </c>
-      <c r="J421" s="6" t="n">
-        <v/>
-      </c>
-      <c r="K421" s="6" t="n">
-        <v/>
-      </c>
-      <c r="L421" s="6" t="n">
-        <v/>
-      </c>
       <c r="M421" s="3" t="inlineStr">
         <is>
           <t>Odd Lay 2x2 (16.50) aprovada na faixa de risco 8.0 - 18.0</t>
         </is>
       </c>
       <c r="N421" s="3" t="n">
-        <v/>
+        <v>95</v>
       </c>
       <c r="O421" s="3" t="n">
-        <v/>
+        <v>12.26</v>
       </c>
     </row>
     <row r="422">
@@ -27052,31 +27126,33 @@
       <c r="G423" s="2" t="n">
         <v>15.5</v>
       </c>
-      <c r="H423" s="6" t="n">
+      <c r="H423" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="I423" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J423" s="4" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="K423" s="4" t="n">
         <v/>
       </c>
-      <c r="I423" s="6" t="n">
+      <c r="L423" s="4" t="n">
         <v/>
       </c>
-      <c r="J423" s="6" t="n">
-        <v/>
-      </c>
-      <c r="K423" s="6" t="n">
-        <v/>
-      </c>
-      <c r="L423" s="6" t="n">
-        <v/>
-      </c>
       <c r="M423" s="3" t="inlineStr">
         <is>
           <t>Odd Lay 2x2 (15.50) aprovada na faixa de risco 8.0 - 18.0</t>
         </is>
       </c>
       <c r="N423" s="3" t="n">
-        <v/>
+        <v>95</v>
       </c>
       <c r="O423" s="3" t="n">
-        <v/>
+        <v>13.1</v>
       </c>
     </row>
     <row r="424">
@@ -27113,31 +27189,33 @@
       <c r="G424" s="2" t="n">
         <v>18</v>
       </c>
-      <c r="H424" s="6" t="n">
+      <c r="H424" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="I424" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J424" s="4" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="K424" s="4" t="n">
         <v/>
       </c>
-      <c r="I424" s="6" t="n">
+      <c r="L424" s="4" t="n">
         <v/>
       </c>
-      <c r="J424" s="6" t="n">
-        <v/>
-      </c>
-      <c r="K424" s="6" t="n">
-        <v/>
-      </c>
-      <c r="L424" s="6" t="n">
-        <v/>
-      </c>
       <c r="M424" s="3" t="inlineStr">
         <is>
           <t>Odd Lay 2x2 (18.00) aprovada na faixa de risco 8.0 - 18.0</t>
         </is>
       </c>
       <c r="N424" s="3" t="n">
-        <v/>
+        <v>95</v>
       </c>
       <c r="O424" s="3" t="n">
-        <v/>
+        <v>11.18</v>
       </c>
     </row>
     <row r="425">
@@ -27804,31 +27882,33 @@
       <c r="G435" s="2" t="n">
         <v>16.5</v>
       </c>
-      <c r="H435" s="6" t="n">
+      <c r="H435" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="I435" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J435" s="4" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="K435" s="4" t="n">
         <v/>
       </c>
-      <c r="I435" s="6" t="n">
+      <c r="L435" s="4" t="n">
         <v/>
       </c>
-      <c r="J435" s="6" t="n">
-        <v/>
-      </c>
-      <c r="K435" s="6" t="n">
-        <v/>
-      </c>
-      <c r="L435" s="6" t="n">
-        <v/>
-      </c>
       <c r="M435" s="3" t="inlineStr">
         <is>
           <t>Odd Lay 2x2 (16.50) aprovada na faixa de risco 8.0 - 18.0</t>
         </is>
       </c>
       <c r="N435" s="3" t="n">
-        <v/>
+        <v>95</v>
       </c>
       <c r="O435" s="3" t="n">
-        <v/>
+        <v>12.26</v>
       </c>
     </row>
     <row r="436">
@@ -27865,31 +27945,33 @@
       <c r="G436" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="H436" s="6" t="n">
+      <c r="H436" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="I436" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="J436" s="4" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="K436" s="4" t="n">
         <v/>
       </c>
-      <c r="I436" s="6" t="n">
+      <c r="L436" s="4" t="n">
         <v/>
       </c>
-      <c r="J436" s="6" t="n">
-        <v/>
-      </c>
-      <c r="K436" s="6" t="n">
-        <v/>
-      </c>
-      <c r="L436" s="6" t="n">
-        <v/>
-      </c>
       <c r="M436" s="3" t="inlineStr">
         <is>
           <t>Odd Lay 2x2 (14.00) aprovada na faixa de risco 8.0 - 18.0</t>
         </is>
       </c>
       <c r="N436" s="3" t="n">
-        <v/>
+        <v>95</v>
       </c>
       <c r="O436" s="3" t="n">
-        <v/>
+        <v>14.62</v>
       </c>
     </row>
     <row r="437">
@@ -27926,31 +28008,33 @@
       <c r="G437" s="2" t="n">
         <v>16.5</v>
       </c>
-      <c r="H437" s="6" t="n">
+      <c r="H437" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I437" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J437" s="4" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="K437" s="4" t="n">
         <v/>
       </c>
-      <c r="I437" s="6" t="n">
+      <c r="L437" s="4" t="n">
         <v/>
       </c>
-      <c r="J437" s="6" t="n">
-        <v/>
-      </c>
-      <c r="K437" s="6" t="n">
-        <v/>
-      </c>
-      <c r="L437" s="6" t="n">
-        <v/>
-      </c>
       <c r="M437" s="3" t="inlineStr">
         <is>
           <t>Odd Lay 2x2 (16.50) aprovada na faixa de risco 8.0 - 18.0</t>
         </is>
       </c>
       <c r="N437" s="3" t="n">
-        <v/>
+        <v>95</v>
       </c>
       <c r="O437" s="3" t="n">
-        <v/>
+        <v>12.26</v>
       </c>
     </row>
     <row r="438">
@@ -27993,9 +28077,7 @@
       <c r="I438" s="6" t="n">
         <v/>
       </c>
-      <c r="J438" s="6" t="n">
-        <v/>
-      </c>
+      <c r="J438" s="6" t="inlineStr"/>
       <c r="K438" s="6" t="n">
         <v/>
       </c>
@@ -28007,12 +28089,8 @@
           <t>Odd Lay 2x2 (15.00) aprovada na faixa de risco 8.0 - 18.0</t>
         </is>
       </c>
-      <c r="N438" s="3" t="n">
-        <v/>
-      </c>
-      <c r="O438" s="3" t="n">
-        <v/>
-      </c>
+      <c r="N438" s="3" t="inlineStr"/>
+      <c r="O438" s="3" t="inlineStr"/>
     </row>
     <row r="439">
       <c r="A439" s="2" t="inlineStr">
@@ -28054,9 +28132,7 @@
       <c r="I439" s="6" t="n">
         <v/>
       </c>
-      <c r="J439" s="6" t="n">
-        <v/>
-      </c>
+      <c r="J439" s="6" t="inlineStr"/>
       <c r="K439" s="6" t="n">
         <v/>
       </c>
@@ -28068,12 +28144,8 @@
           <t>Odd Lay 2x2 (14.00) aprovada na faixa de risco 8.0 - 18.0</t>
         </is>
       </c>
-      <c r="N439" s="3" t="n">
-        <v/>
-      </c>
-      <c r="O439" s="3" t="n">
-        <v/>
-      </c>
+      <c r="N439" s="3" t="inlineStr"/>
+      <c r="O439" s="3" t="inlineStr"/>
     </row>
     <row r="440">
       <c r="A440" s="2" t="inlineStr">
@@ -28115,9 +28187,7 @@
       <c r="I440" s="6" t="n">
         <v/>
       </c>
-      <c r="J440" s="6" t="n">
-        <v/>
-      </c>
+      <c r="J440" s="6" t="inlineStr"/>
       <c r="K440" s="6" t="n">
         <v/>
       </c>
@@ -28129,12 +28199,8 @@
           <t>Odd Lay 2x2 (16.50) aprovada na faixa de risco 8.0 - 18.0</t>
         </is>
       </c>
-      <c r="N440" s="3" t="n">
-        <v/>
-      </c>
-      <c r="O440" s="3" t="n">
-        <v/>
-      </c>
+      <c r="N440" s="3" t="inlineStr"/>
+      <c r="O440" s="3" t="inlineStr"/>
     </row>
     <row r="441">
       <c r="A441" s="2" t="inlineStr">
@@ -28176,9 +28242,7 @@
       <c r="I441" s="6" t="n">
         <v/>
       </c>
-      <c r="J441" s="6" t="n">
-        <v/>
-      </c>
+      <c r="J441" s="6" t="inlineStr"/>
       <c r="K441" s="6" t="n">
         <v/>
       </c>
@@ -28190,12 +28254,8 @@
           <t>Odd Lay 2x2 (15.00) aprovada na faixa de risco 8.0 - 18.0</t>
         </is>
       </c>
-      <c r="N441" s="3" t="n">
-        <v/>
-      </c>
-      <c r="O441" s="3" t="n">
-        <v/>
-      </c>
+      <c r="N441" s="3" t="inlineStr"/>
+      <c r="O441" s="3" t="inlineStr"/>
     </row>
     <row r="442">
       <c r="A442" s="2" t="inlineStr">
@@ -28237,9 +28297,7 @@
       <c r="I442" s="6" t="n">
         <v/>
       </c>
-      <c r="J442" s="6" t="n">
-        <v/>
-      </c>
+      <c r="J442" s="6" t="inlineStr"/>
       <c r="K442" s="6" t="n">
         <v/>
       </c>
@@ -28251,12 +28309,8 @@
           <t>Odd Lay 2x2 (15.00) aprovada na faixa de risco 8.0 - 18.0</t>
         </is>
       </c>
-      <c r="N442" s="3" t="n">
-        <v/>
-      </c>
-      <c r="O442" s="3" t="n">
-        <v/>
-      </c>
+      <c r="N442" s="3" t="inlineStr"/>
+      <c r="O442" s="3" t="inlineStr"/>
     </row>
     <row r="443">
       <c r="A443" s="2" t="inlineStr">
@@ -28298,9 +28352,7 @@
       <c r="I443" s="6" t="n">
         <v/>
       </c>
-      <c r="J443" s="6" t="n">
-        <v/>
-      </c>
+      <c r="J443" s="6" t="inlineStr"/>
       <c r="K443" s="6" t="n">
         <v/>
       </c>
@@ -28312,12 +28364,8 @@
           <t>Odd Lay 2x2 (16.50) aprovada na faixa de risco 8.0 - 18.0</t>
         </is>
       </c>
-      <c r="N443" s="3" t="n">
-        <v/>
-      </c>
-      <c r="O443" s="3" t="n">
-        <v/>
-      </c>
+      <c r="N443" s="3" t="inlineStr"/>
+      <c r="O443" s="3" t="inlineStr"/>
     </row>
     <row r="444">
       <c r="A444" s="2" t="inlineStr">
@@ -28359,9 +28407,7 @@
       <c r="I444" s="6" t="n">
         <v/>
       </c>
-      <c r="J444" s="6" t="n">
-        <v/>
-      </c>
+      <c r="J444" s="6" t="inlineStr"/>
       <c r="K444" s="6" t="n">
         <v/>
       </c>
@@ -28373,12 +28419,8 @@
           <t>Odd Lay 2x2 (13.50) aprovada na faixa de risco 8.0 - 18.0</t>
         </is>
       </c>
-      <c r="N444" s="3" t="n">
-        <v/>
-      </c>
-      <c r="O444" s="3" t="n">
-        <v/>
-      </c>
+      <c r="N444" s="3" t="inlineStr"/>
+      <c r="O444" s="3" t="inlineStr"/>
     </row>
     <row r="445">
       <c r="A445" s="2" t="inlineStr">
@@ -28420,9 +28462,7 @@
       <c r="I445" s="6" t="n">
         <v/>
       </c>
-      <c r="J445" s="6" t="n">
-        <v/>
-      </c>
+      <c r="J445" s="6" t="inlineStr"/>
       <c r="K445" s="6" t="n">
         <v/>
       </c>
@@ -28434,12 +28474,8 @@
           <t>Odd Lay 2x2 (17.00) aprovada na faixa de risco 8.0 - 18.0</t>
         </is>
       </c>
-      <c r="N445" s="3" t="n">
-        <v/>
-      </c>
-      <c r="O445" s="3" t="n">
-        <v/>
-      </c>
+      <c r="N445" s="3" t="inlineStr"/>
+      <c r="O445" s="3" t="inlineStr"/>
     </row>
     <row r="446">
       <c r="A446" s="2" t="inlineStr">
@@ -28481,9 +28517,7 @@
       <c r="I446" s="6" t="n">
         <v/>
       </c>
-      <c r="J446" s="6" t="n">
-        <v/>
-      </c>
+      <c r="J446" s="6" t="inlineStr"/>
       <c r="K446" s="6" t="n">
         <v/>
       </c>
@@ -28495,12 +28529,8 @@
           <t>Odd Lay 2x2 (17.00) aprovada na faixa de risco 8.0 - 18.0</t>
         </is>
       </c>
-      <c r="N446" s="3" t="n">
-        <v/>
-      </c>
-      <c r="O446" s="3" t="n">
-        <v/>
-      </c>
+      <c r="N446" s="3" t="inlineStr"/>
+      <c r="O446" s="3" t="inlineStr"/>
     </row>
     <row r="447">
       <c r="A447" s="2" t="inlineStr">
@@ -28542,9 +28572,7 @@
       <c r="I447" s="6" t="n">
         <v/>
       </c>
-      <c r="J447" s="6" t="n">
-        <v/>
-      </c>
+      <c r="J447" s="6" t="inlineStr"/>
       <c r="K447" s="6" t="n">
         <v/>
       </c>
@@ -28556,12 +28584,8 @@
           <t>Odd Lay 2x2 (15.00) aprovada na faixa de risco 8.0 - 18.0</t>
         </is>
       </c>
-      <c r="N447" s="3" t="n">
-        <v/>
-      </c>
-      <c r="O447" s="3" t="n">
-        <v/>
-      </c>
+      <c r="N447" s="3" t="inlineStr"/>
+      <c r="O447" s="3" t="inlineStr"/>
     </row>
     <row r="448">
       <c r="A448" s="2" t="inlineStr">
@@ -28603,9 +28627,7 @@
       <c r="I448" s="6" t="n">
         <v/>
       </c>
-      <c r="J448" s="6" t="n">
-        <v/>
-      </c>
+      <c r="J448" s="6" t="inlineStr"/>
       <c r="K448" s="6" t="n">
         <v/>
       </c>
@@ -28617,12 +28639,8 @@
           <t>Odd Lay 2x2 (16.50) aprovada na faixa de risco 8.0 - 18.0</t>
         </is>
       </c>
-      <c r="N448" s="3" t="n">
-        <v/>
-      </c>
-      <c r="O448" s="3" t="n">
-        <v/>
-      </c>
+      <c r="N448" s="3" t="inlineStr"/>
+      <c r="O448" s="3" t="inlineStr"/>
     </row>
     <row r="449">
       <c r="A449" s="2" t="inlineStr">
@@ -28664,9 +28682,7 @@
       <c r="I449" s="6" t="n">
         <v/>
       </c>
-      <c r="J449" s="6" t="n">
-        <v/>
-      </c>
+      <c r="J449" s="6" t="inlineStr"/>
       <c r="K449" s="6" t="n">
         <v/>
       </c>
@@ -28678,12 +28694,8 @@
           <t>Odd Lay 2x2 (15.00) aprovada na faixa de risco 8.0 - 18.0</t>
         </is>
       </c>
-      <c r="N449" s="3" t="n">
-        <v/>
-      </c>
-      <c r="O449" s="3" t="n">
-        <v/>
-      </c>
+      <c r="N449" s="3" t="inlineStr"/>
+      <c r="O449" s="3" t="inlineStr"/>
     </row>
     <row r="450">
       <c r="A450" s="2" t="inlineStr">
@@ -28725,9 +28737,7 @@
       <c r="I450" s="6" t="n">
         <v/>
       </c>
-      <c r="J450" s="6" t="n">
-        <v/>
-      </c>
+      <c r="J450" s="6" t="inlineStr"/>
       <c r="K450" s="6" t="n">
         <v/>
       </c>
@@ -28739,12 +28749,8 @@
           <t>Odd Lay 2x2 (14.00) aprovada na faixa de risco 8.0 - 18.0</t>
         </is>
       </c>
-      <c r="N450" s="3" t="n">
-        <v/>
-      </c>
-      <c r="O450" s="3" t="n">
-        <v/>
-      </c>
+      <c r="N450" s="3" t="inlineStr"/>
+      <c r="O450" s="3" t="inlineStr"/>
     </row>
     <row r="451">
       <c r="A451" s="2" t="inlineStr">
@@ -28786,9 +28792,7 @@
       <c r="I451" s="6" t="n">
         <v/>
       </c>
-      <c r="J451" s="6" t="n">
-        <v/>
-      </c>
+      <c r="J451" s="6" t="inlineStr"/>
       <c r="K451" s="6" t="n">
         <v/>
       </c>
@@ -28800,12 +28804,8 @@
           <t>Odd Lay 2x2 (16.50) aprovada na faixa de risco 8.0 - 18.0</t>
         </is>
       </c>
-      <c r="N451" s="3" t="n">
-        <v/>
-      </c>
-      <c r="O451" s="3" t="n">
-        <v/>
-      </c>
+      <c r="N451" s="3" t="inlineStr"/>
+      <c r="O451" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat: completa 449 das 450 partidas na planilha Backtest Lay 2x2 Agosto (427 Greens / 22 Reds - 95.1% Win Rate)
</commit_message>
<xml_diff>
--- a/Backtest_Lay_2x2_Agosto_2026.xlsx
+++ b/Backtest_Lay_2x2_Agosto_2026.xlsx
@@ -28071,26 +28071,34 @@
       <c r="G438" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="H438" s="6" t="n">
+      <c r="H438" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="I438" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="J438" s="4" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="K438" s="4" t="n">
         <v/>
       </c>
-      <c r="I438" s="6" t="n">
+      <c r="L438" s="4" t="n">
         <v/>
       </c>
-      <c r="J438" s="6" t="inlineStr"/>
-      <c r="K438" s="6" t="n">
-        <v/>
-      </c>
-      <c r="L438" s="6" t="n">
-        <v/>
-      </c>
       <c r="M438" s="3" t="inlineStr">
         <is>
           <t>Odd Lay 2x2 (15.00) aprovada na faixa de risco 8.0 - 18.0</t>
         </is>
       </c>
-      <c r="N438" s="3" t="inlineStr"/>
-      <c r="O438" s="3" t="inlineStr"/>
+      <c r="N438" s="3" t="n">
+        <v>95</v>
+      </c>
+      <c r="O438" s="3" t="n">
+        <v>13.57</v>
+      </c>
     </row>
     <row r="439">
       <c r="A439" s="2" t="inlineStr">
@@ -28126,26 +28134,34 @@
       <c r="G439" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="H439" s="6" t="n">
+      <c r="H439" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="I439" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="J439" s="4" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="K439" s="4" t="n">
         <v/>
       </c>
-      <c r="I439" s="6" t="n">
+      <c r="L439" s="4" t="n">
         <v/>
       </c>
-      <c r="J439" s="6" t="inlineStr"/>
-      <c r="K439" s="6" t="n">
-        <v/>
-      </c>
-      <c r="L439" s="6" t="n">
-        <v/>
-      </c>
       <c r="M439" s="3" t="inlineStr">
         <is>
           <t>Odd Lay 2x2 (14.00) aprovada na faixa de risco 8.0 - 18.0</t>
         </is>
       </c>
-      <c r="N439" s="3" t="inlineStr"/>
-      <c r="O439" s="3" t="inlineStr"/>
+      <c r="N439" s="3" t="n">
+        <v>95</v>
+      </c>
+      <c r="O439" s="3" t="n">
+        <v>14.62</v>
+      </c>
     </row>
     <row r="440">
       <c r="A440" s="2" t="inlineStr">
@@ -28181,26 +28197,34 @@
       <c r="G440" s="2" t="n">
         <v>16.5</v>
       </c>
-      <c r="H440" s="6" t="n">
+      <c r="H440" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I440" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="J440" s="4" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="K440" s="4" t="n">
         <v/>
       </c>
-      <c r="I440" s="6" t="n">
+      <c r="L440" s="4" t="n">
         <v/>
       </c>
-      <c r="J440" s="6" t="inlineStr"/>
-      <c r="K440" s="6" t="n">
-        <v/>
-      </c>
-      <c r="L440" s="6" t="n">
-        <v/>
-      </c>
       <c r="M440" s="3" t="inlineStr">
         <is>
           <t>Odd Lay 2x2 (16.50) aprovada na faixa de risco 8.0 - 18.0</t>
         </is>
       </c>
-      <c r="N440" s="3" t="inlineStr"/>
-      <c r="O440" s="3" t="inlineStr"/>
+      <c r="N440" s="3" t="n">
+        <v>95</v>
+      </c>
+      <c r="O440" s="3" t="n">
+        <v>12.26</v>
+      </c>
     </row>
     <row r="441">
       <c r="A441" s="2" t="inlineStr">
@@ -28236,26 +28260,34 @@
       <c r="G441" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="H441" s="6" t="n">
+      <c r="H441" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I441" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J441" s="4" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="K441" s="4" t="n">
         <v/>
       </c>
-      <c r="I441" s="6" t="n">
+      <c r="L441" s="4" t="n">
         <v/>
       </c>
-      <c r="J441" s="6" t="inlineStr"/>
-      <c r="K441" s="6" t="n">
-        <v/>
-      </c>
-      <c r="L441" s="6" t="n">
-        <v/>
-      </c>
       <c r="M441" s="3" t="inlineStr">
         <is>
           <t>Odd Lay 2x2 (15.00) aprovada na faixa de risco 8.0 - 18.0</t>
         </is>
       </c>
-      <c r="N441" s="3" t="inlineStr"/>
-      <c r="O441" s="3" t="inlineStr"/>
+      <c r="N441" s="3" t="n">
+        <v>95</v>
+      </c>
+      <c r="O441" s="3" t="n">
+        <v>13.57</v>
+      </c>
     </row>
     <row r="442">
       <c r="A442" s="2" t="inlineStr">
@@ -28291,26 +28323,34 @@
       <c r="G442" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="H442" s="6" t="n">
+      <c r="H442" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="I442" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J442" s="4" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="K442" s="4" t="n">
         <v/>
       </c>
-      <c r="I442" s="6" t="n">
+      <c r="L442" s="4" t="n">
         <v/>
       </c>
-      <c r="J442" s="6" t="inlineStr"/>
-      <c r="K442" s="6" t="n">
-        <v/>
-      </c>
-      <c r="L442" s="6" t="n">
-        <v/>
-      </c>
       <c r="M442" s="3" t="inlineStr">
         <is>
           <t>Odd Lay 2x2 (15.00) aprovada na faixa de risco 8.0 - 18.0</t>
         </is>
       </c>
-      <c r="N442" s="3" t="inlineStr"/>
-      <c r="O442" s="3" t="inlineStr"/>
+      <c r="N442" s="3" t="n">
+        <v>95</v>
+      </c>
+      <c r="O442" s="3" t="n">
+        <v>13.57</v>
+      </c>
     </row>
     <row r="443">
       <c r="A443" s="2" t="inlineStr">
@@ -28346,26 +28386,34 @@
       <c r="G443" s="2" t="n">
         <v>16.5</v>
       </c>
-      <c r="H443" s="6" t="n">
+      <c r="H443" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="I443" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J443" s="4" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="K443" s="4" t="n">
         <v/>
       </c>
-      <c r="I443" s="6" t="n">
+      <c r="L443" s="4" t="n">
         <v/>
       </c>
-      <c r="J443" s="6" t="inlineStr"/>
-      <c r="K443" s="6" t="n">
-        <v/>
-      </c>
-      <c r="L443" s="6" t="n">
-        <v/>
-      </c>
       <c r="M443" s="3" t="inlineStr">
         <is>
           <t>Odd Lay 2x2 (16.50) aprovada na faixa de risco 8.0 - 18.0</t>
         </is>
       </c>
-      <c r="N443" s="3" t="inlineStr"/>
-      <c r="O443" s="3" t="inlineStr"/>
+      <c r="N443" s="3" t="n">
+        <v>95</v>
+      </c>
+      <c r="O443" s="3" t="n">
+        <v>12.26</v>
+      </c>
     </row>
     <row r="444">
       <c r="A444" s="2" t="inlineStr">
@@ -28401,26 +28449,34 @@
       <c r="G444" s="2" t="n">
         <v>13.5</v>
       </c>
-      <c r="H444" s="6" t="n">
+      <c r="H444" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="I444" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="J444" s="4" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="K444" s="4" t="n">
         <v/>
       </c>
-      <c r="I444" s="6" t="n">
+      <c r="L444" s="4" t="n">
         <v/>
       </c>
-      <c r="J444" s="6" t="inlineStr"/>
-      <c r="K444" s="6" t="n">
-        <v/>
-      </c>
-      <c r="L444" s="6" t="n">
-        <v/>
-      </c>
       <c r="M444" s="3" t="inlineStr">
         <is>
           <t>Odd Lay 2x2 (13.50) aprovada na faixa de risco 8.0 - 18.0</t>
         </is>
       </c>
-      <c r="N444" s="3" t="inlineStr"/>
-      <c r="O444" s="3" t="inlineStr"/>
+      <c r="N444" s="3" t="n">
+        <v>95</v>
+      </c>
+      <c r="O444" s="3" t="n">
+        <v>15.2</v>
+      </c>
     </row>
     <row r="445">
       <c r="A445" s="2" t="inlineStr">
@@ -28456,26 +28512,34 @@
       <c r="G445" s="2" t="n">
         <v>17</v>
       </c>
-      <c r="H445" s="6" t="n">
+      <c r="H445" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="I445" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J445" s="4" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="K445" s="4" t="n">
         <v/>
       </c>
-      <c r="I445" s="6" t="n">
+      <c r="L445" s="4" t="n">
         <v/>
       </c>
-      <c r="J445" s="6" t="inlineStr"/>
-      <c r="K445" s="6" t="n">
-        <v/>
-      </c>
-      <c r="L445" s="6" t="n">
-        <v/>
-      </c>
       <c r="M445" s="3" t="inlineStr">
         <is>
           <t>Odd Lay 2x2 (17.00) aprovada na faixa de risco 8.0 - 18.0</t>
         </is>
       </c>
-      <c r="N445" s="3" t="inlineStr"/>
-      <c r="O445" s="3" t="inlineStr"/>
+      <c r="N445" s="3" t="n">
+        <v>95</v>
+      </c>
+      <c r="O445" s="3" t="n">
+        <v>11.88</v>
+      </c>
     </row>
     <row r="446">
       <c r="A446" s="2" t="inlineStr">
@@ -28511,26 +28575,34 @@
       <c r="G446" s="2" t="n">
         <v>17</v>
       </c>
-      <c r="H446" s="6" t="n">
+      <c r="H446" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="I446" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="J446" s="4" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="K446" s="4" t="n">
         <v/>
       </c>
-      <c r="I446" s="6" t="n">
+      <c r="L446" s="4" t="n">
         <v/>
       </c>
-      <c r="J446" s="6" t="inlineStr"/>
-      <c r="K446" s="6" t="n">
-        <v/>
-      </c>
-      <c r="L446" s="6" t="n">
-        <v/>
-      </c>
       <c r="M446" s="3" t="inlineStr">
         <is>
           <t>Odd Lay 2x2 (17.00) aprovada na faixa de risco 8.0 - 18.0</t>
         </is>
       </c>
-      <c r="N446" s="3" t="inlineStr"/>
-      <c r="O446" s="3" t="inlineStr"/>
+      <c r="N446" s="3" t="n">
+        <v>95</v>
+      </c>
+      <c r="O446" s="3" t="n">
+        <v>11.88</v>
+      </c>
     </row>
     <row r="447">
       <c r="A447" s="2" t="inlineStr">
@@ -28566,26 +28638,34 @@
       <c r="G447" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="H447" s="6" t="n">
+      <c r="H447" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I447" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J447" s="4" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="K447" s="4" t="n">
         <v/>
       </c>
-      <c r="I447" s="6" t="n">
+      <c r="L447" s="4" t="n">
         <v/>
       </c>
-      <c r="J447" s="6" t="inlineStr"/>
-      <c r="K447" s="6" t="n">
-        <v/>
-      </c>
-      <c r="L447" s="6" t="n">
-        <v/>
-      </c>
       <c r="M447" s="3" t="inlineStr">
         <is>
           <t>Odd Lay 2x2 (15.00) aprovada na faixa de risco 8.0 - 18.0</t>
         </is>
       </c>
-      <c r="N447" s="3" t="inlineStr"/>
-      <c r="O447" s="3" t="inlineStr"/>
+      <c r="N447" s="3" t="n">
+        <v>95</v>
+      </c>
+      <c r="O447" s="3" t="n">
+        <v>13.57</v>
+      </c>
     </row>
     <row r="448">
       <c r="A448" s="2" t="inlineStr">
@@ -28621,26 +28701,34 @@
       <c r="G448" s="2" t="n">
         <v>16.5</v>
       </c>
-      <c r="H448" s="6" t="n">
+      <c r="H448" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="I448" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="J448" s="5" t="inlineStr">
+        <is>
+          <t>RED</t>
+        </is>
+      </c>
+      <c r="K448" s="5" t="n">
         <v/>
       </c>
-      <c r="I448" s="6" t="n">
+      <c r="L448" s="5" t="n">
         <v/>
       </c>
-      <c r="J448" s="6" t="inlineStr"/>
-      <c r="K448" s="6" t="n">
-        <v/>
-      </c>
-      <c r="L448" s="6" t="n">
-        <v/>
-      </c>
       <c r="M448" s="3" t="inlineStr">
         <is>
           <t>Odd Lay 2x2 (16.50) aprovada na faixa de risco 8.0 - 18.0</t>
         </is>
       </c>
-      <c r="N448" s="3" t="inlineStr"/>
-      <c r="O448" s="3" t="inlineStr"/>
+      <c r="N448" s="3" t="n">
+        <v>-1550</v>
+      </c>
+      <c r="O448" s="3" t="n">
+        <v>-200</v>
+      </c>
     </row>
     <row r="449">
       <c r="A449" s="2" t="inlineStr">
@@ -28676,26 +28764,34 @@
       <c r="G449" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="H449" s="6" t="n">
+      <c r="H449" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="I449" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J449" s="4" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="K449" s="4" t="n">
         <v/>
       </c>
-      <c r="I449" s="6" t="n">
+      <c r="L449" s="4" t="n">
         <v/>
       </c>
-      <c r="J449" s="6" t="inlineStr"/>
-      <c r="K449" s="6" t="n">
-        <v/>
-      </c>
-      <c r="L449" s="6" t="n">
-        <v/>
-      </c>
       <c r="M449" s="3" t="inlineStr">
         <is>
           <t>Odd Lay 2x2 (15.00) aprovada na faixa de risco 8.0 - 18.0</t>
         </is>
       </c>
-      <c r="N449" s="3" t="inlineStr"/>
-      <c r="O449" s="3" t="inlineStr"/>
+      <c r="N449" s="3" t="n">
+        <v>95</v>
+      </c>
+      <c r="O449" s="3" t="n">
+        <v>13.57</v>
+      </c>
     </row>
     <row r="450">
       <c r="A450" s="2" t="inlineStr">
@@ -28731,26 +28827,34 @@
       <c r="G450" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="H450" s="6" t="n">
+      <c r="H450" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="I450" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J450" s="4" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="K450" s="4" t="n">
         <v/>
       </c>
-      <c r="I450" s="6" t="n">
+      <c r="L450" s="4" t="n">
         <v/>
       </c>
-      <c r="J450" s="6" t="inlineStr"/>
-      <c r="K450" s="6" t="n">
-        <v/>
-      </c>
-      <c r="L450" s="6" t="n">
-        <v/>
-      </c>
       <c r="M450" s="3" t="inlineStr">
         <is>
           <t>Odd Lay 2x2 (14.00) aprovada na faixa de risco 8.0 - 18.0</t>
         </is>
       </c>
-      <c r="N450" s="3" t="inlineStr"/>
-      <c r="O450" s="3" t="inlineStr"/>
+      <c r="N450" s="3" t="n">
+        <v>95</v>
+      </c>
+      <c r="O450" s="3" t="n">
+        <v>14.62</v>
+      </c>
     </row>
     <row r="451">
       <c r="A451" s="2" t="inlineStr">

</xml_diff>